<commit_message>
implemented the embedded image in excel
</commit_message>
<xml_diff>
--- a/outputs/08_06_2026.xlsx
+++ b/outputs/08_06_2026.xlsx
@@ -1,91 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Security_system\outputs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8459FECB-4A59-4814-BB90-AFC6DCA682CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>color</t>
-  </si>
-  <si>
-    <t>plate</t>
-  </si>
-  <si>
-    <t>entry_time</t>
-  </si>
-  <si>
-    <t>vehicle_image</t>
-  </si>
-  <si>
-    <t>plate_image</t>
-  </si>
-  <si>
-    <t>debug_plate_image</t>
-  </si>
-  <si>
-    <t>car</t>
-  </si>
-  <si>
-    <t>BLUE</t>
-  </si>
-  <si>
-    <t>IN30A00707</t>
-  </si>
-  <si>
-    <t>2026-06-08_20-42-37</t>
-  </si>
-  <si>
-    <t>snapshots/vehicle_1.jpg</t>
-  </si>
-  <si>
-    <t>snapshots/plate_1.jpg</t>
-  </si>
-  <si>
-    <t>snapshots/debug_plate_1.jpg</t>
-  </si>
-  <si>
-    <t>2026-06-08_20-44-08</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -104,22 +46,161 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2305050" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1419225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -406,96 +487,170 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="37.5546875" customWidth="1"/>
-    <col min="5" max="5" width="29.5546875" customWidth="1"/>
-    <col min="6" max="6" width="27.77734375" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="29" customWidth="1"/>
+    <col width="37.5546875" customWidth="1" min="4" max="4"/>
+    <col width="29.5546875" customWidth="1" min="5" max="5"/>
+    <col width="27.77734375" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>plate</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>entry_time</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>vehicle_image</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>plate_image</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>debug_plate_image</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-06-08_20-42-37</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>snapshots/vehicle_1.jpg</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>snapshots/plate_1.jpg</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>snapshots/debug_plate_1.jpg</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="3">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-06-08_20-44-08</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>snapshots/vehicle_1.jpg</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>snapshots/plate_1.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>snapshots/debug_plate_1.jpg</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="4" ht="111" customHeight="1">
+      <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-06-08_21-17-07</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
embedded image fitted inside the cell
</commit_message>
<xml_diff>
--- a/outputs/08_06_2026.xlsx
+++ b/outputs/08_06_2026.xlsx
@@ -146,6 +146,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -171,6 +174,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -190,6 +196,84 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2305050" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1419225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -492,14 +576,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="37.5546875" customWidth="1" min="4" max="4"/>
     <col width="29.5546875" customWidth="1" min="5" max="5"/>
-    <col width="27.77734375" customWidth="1" min="6" max="6"/>
+    <col width="35.88" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="46.8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -646,6 +730,31 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>2026-06-08_21-17-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="135" customHeight="1">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-06-08_21-21-37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
remove debuged_plate_image column from report
</commit_message>
<xml_diff>
--- a/outputs/08_06_2026.xlsx
+++ b/outputs/08_06_2026.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -129,7 +130,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2305050" cy="1714500"/>
@@ -146,9 +147,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -157,7 +155,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1143000" cy="533400"/>
@@ -168,112 +166,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3048000" cy="1419225"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2305050" cy="1714500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1143000" cy="533400"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3048000" cy="1419225"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -576,14 +468,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37.5546875" customWidth="1" min="4" max="4"/>
-    <col width="29.5546875" customWidth="1" min="5" max="5"/>
     <col width="35.88" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="46.8" customWidth="1" min="8" max="8"/>
+    <col width="18.8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -622,13 +511,8 @@
           <t>plate_image</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>debug_plate_image</t>
-        </is>
-      </c>
     </row>
-    <row r="2">
+    <row r="2" ht="135" customHeight="1">
       <c r="A2" t="n">
         <v>1</v>
       </c>
@@ -649,112 +533,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-08_20-42-37</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>snapshots/vehicle_1.jpg</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>snapshots/plate_1.jpg</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>snapshots/debug_plate_1.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>car</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>IN30A00707</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-06-08_20-44-08</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>snapshots/vehicle_1.jpg</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>snapshots/plate_1.jpg</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>snapshots/debug_plate_1.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="111" customHeight="1">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>car</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>IN30A00707</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-06-08_21-17-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="135" customHeight="1">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>car</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>IN30A00707</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-06-08_21-21-37</t>
+          <t>2026-06-08_21-25-53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
date format to 12 hour format
</commit_message>
<xml_diff>
--- a/outputs/08_06_2026.xlsx
+++ b/outputs/08_06_2026.xlsx
@@ -147,6 +147,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -166,6 +169,59 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2305050" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -468,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35.88" customWidth="1" min="6" max="6"/>
@@ -537,6 +593,31 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="135" customHeight="1">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>08:06:2026  09:32:28  PM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
date format with DD monthinwords YYYY
</commit_message>
<xml_diff>
--- a/outputs/08_06_2026.xlsx
+++ b/outputs/08_06_2026.xlsx
@@ -203,6 +203,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -222,6 +225,59 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2305050" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -524,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35.88" customWidth="1" min="6" max="6"/>
@@ -618,6 +674,31 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="135" customHeight="1">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IN30A00707</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>08 June 2026  09:37:56  PM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>